<commit_message>
Update network simulation results files
</commit_message>
<xml_diff>
--- a/analysis/network_simulation_results/Stats checkpoints.xlsx
+++ b/analysis/network_simulation_results/Stats checkpoints.xlsx
@@ -14,11 +14,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={b775ba41-8e92-4728-ad72-efa5b64cae78}</author>
-    <author>tc={ddc75ed5-39b9-4341-b6b6-5569c1089c7a}</author>
+    <author>tc={d1881085-9965-4963-b085-6892a0a043d0}</author>
+    <author>tc={ef1411ca-7577-4a58-b959-185a64fbe668}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{b775ba41-8e92-4728-ad72-efa5b64cae78}" ref="A6">
+    <comment authorId="0" xr:uid="{d1881085-9965-4963-b085-6892a0a043d0}" ref="A6">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -27,7 +27,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{ddc75ed5-39b9-4341-b6b6-5569c1089c7a}" ref="D6">
+    <comment authorId="1" xr:uid="{ef1411ca-7577-4a58-b959-185a64fbe668}" ref="D6">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -778,7 +778,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Anastasiya Danilenka" id="{12282387-9436-42df-99c6-da7c601d80d2}" providerId="google-sheets"/>
+  <x18tc:person displayName="Anastasiya Danilenka" id="{3371f989-3167-4012-b6e6-0dc66ffe438f}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -978,10 +978,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="D6" dT="2026-05-07T11:23:26.00" personId="{12282387-9436-42df-99c6-da7c601d80d2}" id="{ddc75ed5-39b9-4341-b6b6-5569c1089c7a}" done="0">
+  <x18tc:threadedComment ref="D6" dT="2026-05-07T11:23:26.00" personId="{3371f989-3167-4012-b6e6-0dc66ffe438f}" id="{ef1411ca-7577-4a58-b959-185a64fbe668}" done="0">
     <x18tc:text xml:space="preserve">estimation based on estimated avg cluster ingestion speed</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A6" dT="2026-05-07T11:22:58.00" personId="{12282387-9436-42df-99c6-da7c601d80d2}" id="{b775ba41-8e92-4728-ad72-efa5b64cae78}" done="0">
+  <x18tc:threadedComment ref="A6" dT="2026-05-07T11:22:58.00" personId="{3371f989-3167-4012-b6e6-0dc66ffe438f}" id="{d1881085-9965-4963-b085-6892a0a043d0}" done="0">
     <x18tc:text xml:space="preserve">query instances experienced issues, so ingestion run was stopped, query instances were restarted, run was continued, numbers are taken after queries restart</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -54023,7 +54023,7 @@
         <v>1.0</v>
       </c>
       <c r="B12" s="91">
-        <v>63769.0</v>
+        <v>0.0</v>
       </c>
       <c r="C12" s="91">
         <v>0.0</v>
@@ -54158,7 +54158,7 @@
         <v>2.0</v>
       </c>
       <c r="B13" s="91">
-        <v>98489.0</v>
+        <v>0.0</v>
       </c>
       <c r="C13" s="91">
         <v>0.0</v>
@@ -54293,7 +54293,7 @@
         <v>3.0</v>
       </c>
       <c r="B14" s="91">
-        <v>153195.0</v>
+        <v>0.0</v>
       </c>
       <c r="C14" s="91">
         <v>0.0</v>
@@ -54428,7 +54428,7 @@
         <v>4.0</v>
       </c>
       <c r="B15" s="93">
-        <v>158614.0</v>
+        <v>0.0</v>
       </c>
       <c r="C15" s="93">
         <v>0.0</v>

</xml_diff>